<commit_message>
feat: gestion de series repetitivas y vinculacion de movimientos con pasivos
</commit_message>
<xml_diff>
--- a/00. Balance 2026 IA.xlsx
+++ b/00. Balance 2026 IA.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\01. PERSONAL\01. ECONOMIA\00. GESTION\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jbasterrika\Desktop\CODING\PIXDEMIA WEB\Finanzas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56F43F81-11DB-4D57-9816-9275E3703D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8736218C-3209-42CD-A0C9-8A3B0AF14F9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AÑO 2026" sheetId="1" r:id="rId1"/>
@@ -7707,156 +7707,156 @@
     <xf numFmtId="0" fontId="4" fillId="71" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="168" fontId="4" fillId="71" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="168" fontId="4" fillId="71" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="13" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="20" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="31" fillId="20" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="20" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="20" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="20" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="16" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="14" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="13" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="43" fillId="7" borderId="3" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="3" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="4" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="70" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="43" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="53" fillId="3" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="59" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -9534,11 +9534,11 @@
         <f>R15-R9</f>
         <v>-2464.3499999999985</v>
       </c>
-      <c r="T15" s="1125">
+      <c r="T15" s="1122">
         <f>S15+S16+S17</f>
         <v>154.77000000000771</v>
       </c>
-      <c r="U15" s="1126">
+      <c r="U15" s="1123">
         <f>T18+T15</f>
         <v>989.21000000000276</v>
       </c>
@@ -9607,8 +9607,8 @@
         <f>R16-R10</f>
         <v>364.45000000000437</v>
       </c>
-      <c r="T16" s="1125"/>
-      <c r="U16" s="1126"/>
+      <c r="T16" s="1122"/>
+      <c r="U16" s="1123"/>
     </row>
     <row r="17" spans="1:21" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="66"/>
@@ -9674,8 +9674,8 @@
         <f>R17-R11</f>
         <v>2254.6700000000019</v>
       </c>
-      <c r="T17" s="1125"/>
-      <c r="U17" s="1126"/>
+      <c r="T17" s="1122"/>
+      <c r="U17" s="1123"/>
     </row>
     <row r="18" spans="1:21" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="67"/>
@@ -9741,11 +9741,11 @@
         <f>R18-R12</f>
         <v>417.21999999999753</v>
       </c>
-      <c r="T18" s="1127">
+      <c r="T18" s="1124">
         <f>S18+S19</f>
         <v>834.43999999999505</v>
       </c>
-      <c r="U18" s="1126"/>
+      <c r="U18" s="1123"/>
     </row>
     <row r="19" spans="1:21" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A19" s="67"/>
@@ -9811,8 +9811,8 @@
         <f>R19-R13</f>
         <v>417.21999999999753</v>
       </c>
-      <c r="T19" s="1127"/>
-      <c r="U19" s="1126"/>
+      <c r="T19" s="1124"/>
+      <c r="U19" s="1123"/>
     </row>
     <row r="20" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="F20" s="19">
@@ -9865,57 +9865,57 @@
       </c>
     </row>
     <row r="21" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1130" t="s">
+      <c r="A21" s="1117" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="1131"/>
-      <c r="C21" s="1130" t="s">
+      <c r="B21" s="1118"/>
+      <c r="C21" s="1117" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="1130" t="s">
+      <c r="D21" s="1117" t="s">
         <v>36</v>
       </c>
-      <c r="E21" s="1132" t="s">
+      <c r="E21" s="1119" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="1128">
+      <c r="F21" s="1125">
         <v>2026</v>
       </c>
-      <c r="G21" s="1128"/>
-      <c r="H21" s="1128"/>
-      <c r="I21" s="1128"/>
-      <c r="J21" s="1128"/>
-      <c r="K21" s="1128"/>
-      <c r="L21" s="1128"/>
-      <c r="M21" s="1128"/>
-      <c r="N21" s="1128"/>
-      <c r="O21" s="1128"/>
-      <c r="P21" s="1128"/>
-      <c r="Q21" s="1128"/>
-      <c r="R21" s="1129" t="s">
+      <c r="G21" s="1125"/>
+      <c r="H21" s="1125"/>
+      <c r="I21" s="1125"/>
+      <c r="J21" s="1125"/>
+      <c r="K21" s="1125"/>
+      <c r="L21" s="1125"/>
+      <c r="M21" s="1125"/>
+      <c r="N21" s="1125"/>
+      <c r="O21" s="1125"/>
+      <c r="P21" s="1125"/>
+      <c r="Q21" s="1125"/>
+      <c r="R21" s="1126" t="s">
         <v>38</v>
       </c>
       <c r="S21" s="53"/>
     </row>
     <row r="22" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1130"/>
-      <c r="B22" s="1131"/>
-      <c r="C22" s="1130"/>
-      <c r="D22" s="1130"/>
-      <c r="E22" s="1132"/>
-      <c r="F22" s="1128"/>
-      <c r="G22" s="1128"/>
-      <c r="H22" s="1128"/>
-      <c r="I22" s="1128"/>
-      <c r="J22" s="1128"/>
-      <c r="K22" s="1128"/>
-      <c r="L22" s="1128"/>
-      <c r="M22" s="1128"/>
-      <c r="N22" s="1128"/>
-      <c r="O22" s="1128"/>
-      <c r="P22" s="1128"/>
-      <c r="Q22" s="1128"/>
-      <c r="R22" s="1129"/>
+      <c r="A22" s="1117"/>
+      <c r="B22" s="1118"/>
+      <c r="C22" s="1117"/>
+      <c r="D22" s="1117"/>
+      <c r="E22" s="1119"/>
+      <c r="F22" s="1125"/>
+      <c r="G22" s="1125"/>
+      <c r="H22" s="1125"/>
+      <c r="I22" s="1125"/>
+      <c r="J22" s="1125"/>
+      <c r="K22" s="1125"/>
+      <c r="L22" s="1125"/>
+      <c r="M22" s="1125"/>
+      <c r="N22" s="1125"/>
+      <c r="O22" s="1125"/>
+      <c r="P22" s="1125"/>
+      <c r="Q22" s="1125"/>
+      <c r="R22" s="1126"/>
     </row>
     <row r="23" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="81"/>
@@ -9967,20 +9967,20 @@
       <c r="C24" s="86"/>
       <c r="D24" s="86"/>
       <c r="E24" s="86"/>
-      <c r="F24" s="1123" t="s">
+      <c r="F24" s="1120" t="s">
         <v>51</v>
       </c>
-      <c r="G24" s="1123"/>
-      <c r="H24" s="1123"/>
-      <c r="I24" s="1123"/>
-      <c r="J24" s="1123"/>
-      <c r="K24" s="1123"/>
-      <c r="L24" s="1123"/>
-      <c r="M24" s="1123"/>
-      <c r="N24" s="1123"/>
-      <c r="O24" s="1123"/>
-      <c r="P24" s="1123"/>
-      <c r="Q24" s="1123"/>
+      <c r="G24" s="1120"/>
+      <c r="H24" s="1120"/>
+      <c r="I24" s="1120"/>
+      <c r="J24" s="1120"/>
+      <c r="K24" s="1120"/>
+      <c r="L24" s="1120"/>
+      <c r="M24" s="1120"/>
+      <c r="N24" s="1120"/>
+      <c r="O24" s="1120"/>
+      <c r="P24" s="1120"/>
+      <c r="Q24" s="1120"/>
       <c r="R24" s="87"/>
     </row>
     <row r="25" spans="1:21" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -10930,20 +10930,20 @@
       <c r="C47" s="127"/>
       <c r="D47" s="127"/>
       <c r="E47" s="127"/>
-      <c r="F47" s="1124" t="s">
+      <c r="F47" s="1121" t="s">
         <v>66</v>
       </c>
-      <c r="G47" s="1124"/>
-      <c r="H47" s="1124"/>
-      <c r="I47" s="1124"/>
-      <c r="J47" s="1124"/>
-      <c r="K47" s="1124"/>
-      <c r="L47" s="1124"/>
-      <c r="M47" s="1124"/>
-      <c r="N47" s="1124"/>
-      <c r="O47" s="1124"/>
-      <c r="P47" s="1124"/>
-      <c r="Q47" s="1124"/>
+      <c r="G47" s="1121"/>
+      <c r="H47" s="1121"/>
+      <c r="I47" s="1121"/>
+      <c r="J47" s="1121"/>
+      <c r="K47" s="1121"/>
+      <c r="L47" s="1121"/>
+      <c r="M47" s="1121"/>
+      <c r="N47" s="1121"/>
+      <c r="O47" s="1121"/>
+      <c r="P47" s="1121"/>
+      <c r="Q47" s="1121"/>
       <c r="R47" s="128"/>
     </row>
     <row r="48" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.2">
@@ -15699,11 +15699,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="E21:E22"/>
     <mergeCell ref="F24:Q24"/>
     <mergeCell ref="F47:Q47"/>
     <mergeCell ref="T15:T17"/>
@@ -15711,6 +15706,11 @@
     <mergeCell ref="T18:T19"/>
     <mergeCell ref="F21:Q22"/>
     <mergeCell ref="R21:R22"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="E21:E22"/>
   </mergeCells>
   <conditionalFormatting sqref="F151:Q151">
     <cfRule type="colorScale" priority="8">
@@ -15873,108 +15873,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1122" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1116" t="s">
+      <c r="A1" s="1127" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1128" t="s">
         <v>39</v>
       </c>
-      <c r="C1" s="1116"/>
-      <c r="D1" s="1116"/>
-      <c r="E1" s="1116"/>
-      <c r="F1" s="1115"/>
+      <c r="C1" s="1128"/>
+      <c r="D1" s="1128"/>
+      <c r="E1" s="1128"/>
+      <c r="F1" s="1129"/>
       <c r="G1" s="838"/>
-      <c r="H1" s="1114" t="s">
+      <c r="H1" s="1130" t="s">
         <v>40</v>
       </c>
-      <c r="I1" s="1114"/>
-      <c r="J1" s="1114"/>
-      <c r="K1" s="1114"/>
-      <c r="L1" s="1114"/>
+      <c r="I1" s="1130"/>
+      <c r="J1" s="1130"/>
+      <c r="K1" s="1130"/>
+      <c r="L1" s="1130"/>
       <c r="M1" s="411"/>
-      <c r="N1" s="1116" t="s">
+      <c r="N1" s="1128" t="s">
         <v>41</v>
       </c>
-      <c r="O1" s="1116"/>
-      <c r="P1" s="1116"/>
-      <c r="Q1" s="1116"/>
-      <c r="R1" s="1116"/>
+      <c r="O1" s="1128"/>
+      <c r="P1" s="1128"/>
+      <c r="Q1" s="1128"/>
+      <c r="R1" s="1128"/>
       <c r="S1" s="838"/>
-      <c r="T1" s="1114" t="s">
+      <c r="T1" s="1130" t="s">
         <v>42</v>
       </c>
-      <c r="U1" s="1114"/>
-      <c r="V1" s="1114"/>
-      <c r="W1" s="1114"/>
-      <c r="X1" s="1114"/>
+      <c r="U1" s="1130"/>
+      <c r="V1" s="1130"/>
+      <c r="W1" s="1130"/>
+      <c r="X1" s="1130"/>
       <c r="Y1" s="411"/>
-      <c r="Z1" s="1116" t="s">
+      <c r="Z1" s="1128" t="s">
         <v>43</v>
       </c>
-      <c r="AA1" s="1116"/>
-      <c r="AB1" s="1116"/>
-      <c r="AC1" s="1116"/>
-      <c r="AD1" s="1116"/>
+      <c r="AA1" s="1128"/>
+      <c r="AB1" s="1128"/>
+      <c r="AC1" s="1128"/>
+      <c r="AD1" s="1128"/>
       <c r="AE1" s="838"/>
-      <c r="AF1" s="1118" t="s">
+      <c r="AF1" s="1131" t="s">
         <v>44</v>
       </c>
-      <c r="AG1" s="1118"/>
-      <c r="AH1" s="1118"/>
-      <c r="AI1" s="1118"/>
-      <c r="AJ1" s="1118"/>
+      <c r="AG1" s="1131"/>
+      <c r="AH1" s="1131"/>
+      <c r="AI1" s="1131"/>
+      <c r="AJ1" s="1131"/>
       <c r="AK1" s="411"/>
-      <c r="AL1" s="1118" t="s">
+      <c r="AL1" s="1131" t="s">
         <v>45</v>
       </c>
-      <c r="AM1" s="1118"/>
-      <c r="AN1" s="1118"/>
-      <c r="AO1" s="1118"/>
-      <c r="AP1" s="1118"/>
+      <c r="AM1" s="1131"/>
+      <c r="AN1" s="1131"/>
+      <c r="AO1" s="1131"/>
+      <c r="AP1" s="1131"/>
       <c r="AQ1" s="838"/>
-      <c r="AR1" s="1114" t="s">
+      <c r="AR1" s="1130" t="s">
         <v>46</v>
       </c>
-      <c r="AS1" s="1114"/>
-      <c r="AT1" s="1114"/>
-      <c r="AU1" s="1114"/>
-      <c r="AV1" s="1114"/>
+      <c r="AS1" s="1130"/>
+      <c r="AT1" s="1130"/>
+      <c r="AU1" s="1130"/>
+      <c r="AV1" s="1130"/>
       <c r="AW1" s="411"/>
-      <c r="AX1" s="1118" t="s">
+      <c r="AX1" s="1131" t="s">
         <v>47</v>
       </c>
-      <c r="AY1" s="1118"/>
-      <c r="AZ1" s="1118"/>
-      <c r="BA1" s="1118"/>
-      <c r="BB1" s="1118"/>
+      <c r="AY1" s="1131"/>
+      <c r="AZ1" s="1131"/>
+      <c r="BA1" s="1131"/>
+      <c r="BB1" s="1131"/>
       <c r="BC1" s="838"/>
-      <c r="BD1" s="1114" t="s">
+      <c r="BD1" s="1130" t="s">
         <v>48</v>
       </c>
-      <c r="BE1" s="1114"/>
-      <c r="BF1" s="1114"/>
-      <c r="BG1" s="1114"/>
-      <c r="BH1" s="1114"/>
+      <c r="BE1" s="1130"/>
+      <c r="BF1" s="1130"/>
+      <c r="BG1" s="1130"/>
+      <c r="BH1" s="1130"/>
       <c r="BI1" s="411"/>
-      <c r="BJ1" s="1115" t="s">
+      <c r="BJ1" s="1129" t="s">
         <v>49</v>
       </c>
-      <c r="BK1" s="1115"/>
-      <c r="BL1" s="1115"/>
-      <c r="BM1" s="1115"/>
-      <c r="BN1" s="1115"/>
+      <c r="BK1" s="1129"/>
+      <c r="BL1" s="1129"/>
+      <c r="BM1" s="1129"/>
+      <c r="BN1" s="1129"/>
       <c r="BO1" s="838"/>
-      <c r="BP1" s="1114" t="s">
+      <c r="BP1" s="1130" t="s">
         <v>50</v>
       </c>
-      <c r="BQ1" s="1114"/>
-      <c r="BR1" s="1114"/>
-      <c r="BS1" s="1114"/>
-      <c r="BT1" s="1114"/>
+      <c r="BQ1" s="1130"/>
+      <c r="BR1" s="1130"/>
+      <c r="BS1" s="1130"/>
+      <c r="BT1" s="1130"/>
       <c r="BU1" s="411"/>
     </row>
     <row r="2" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1122"/>
+      <c r="A2" s="1127"/>
       <c r="B2" s="854" t="s">
         <v>175</v>
       </c>
@@ -16193,7 +16193,7 @@
       </c>
     </row>
     <row r="3" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1122"/>
+      <c r="A3" s="1127"/>
       <c r="B3" s="846">
         <v>10</v>
       </c>
@@ -16312,7 +16312,7 @@
       <c r="BU3" s="849"/>
     </row>
     <row r="4" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1122"/>
+      <c r="A4" s="1127"/>
       <c r="B4" s="362">
         <v>46038</v>
       </c>
@@ -16453,7 +16453,7 @@
       <c r="BU4" s="365"/>
     </row>
     <row r="5" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1122"/>
+      <c r="A5" s="1127"/>
       <c r="B5" s="378">
         <v>46038</v>
       </c>
@@ -16590,7 +16590,7 @@
       <c r="BU5" s="365"/>
     </row>
     <row r="6" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="1122"/>
+      <c r="A6" s="1127"/>
       <c r="B6" s="362">
         <v>46041</v>
       </c>
@@ -16717,7 +16717,7 @@
       <c r="BU6" s="365"/>
     </row>
     <row r="7" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1122"/>
+      <c r="A7" s="1127"/>
       <c r="B7" s="362">
         <v>46048</v>
       </c>
@@ -16826,7 +16826,7 @@
       <c r="BU7" s="365"/>
     </row>
     <row r="8" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1122"/>
+      <c r="A8" s="1127"/>
       <c r="B8" s="382"/>
       <c r="C8" s="363"/>
       <c r="D8" s="363"/>
@@ -16921,7 +16921,7 @@
       <c r="BU8" s="365"/>
     </row>
     <row r="9" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1122"/>
+      <c r="A9" s="1127"/>
       <c r="B9" s="382"/>
       <c r="C9" s="363"/>
       <c r="D9" s="363"/>
@@ -17004,7 +17004,7 @@
       <c r="BU9" s="365"/>
     </row>
     <row r="10" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1122"/>
+      <c r="A10" s="1127"/>
       <c r="B10" s="382"/>
       <c r="C10" s="363"/>
       <c r="D10" s="363"/>
@@ -17079,7 +17079,7 @@
       <c r="BU10" s="365"/>
     </row>
     <row r="11" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1122"/>
+      <c r="A11" s="1127"/>
       <c r="B11" s="382"/>
       <c r="C11" s="363"/>
       <c r="D11" s="363"/>
@@ -17154,7 +17154,7 @@
       <c r="BU11" s="365"/>
     </row>
     <row r="12" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1122"/>
+      <c r="A12" s="1127"/>
       <c r="B12" s="382"/>
       <c r="C12" s="363"/>
       <c r="D12" s="363"/>
@@ -17229,7 +17229,7 @@
       <c r="BU12" s="365"/>
     </row>
     <row r="13" spans="1:73" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1122"/>
+      <c r="A13" s="1127"/>
       <c r="B13" s="382"/>
       <c r="C13" s="363"/>
       <c r="D13" s="363"/>
@@ -17304,7 +17304,7 @@
       <c r="BU13" s="365"/>
     </row>
     <row r="14" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="1122"/>
+      <c r="A14" s="1127"/>
       <c r="B14" s="382"/>
       <c r="C14" s="363"/>
       <c r="D14" s="363"/>
@@ -17391,7 +17391,7 @@
       <c r="BU14" s="365"/>
     </row>
     <row r="15" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1122"/>
+      <c r="A15" s="1127"/>
       <c r="B15" s="382"/>
       <c r="C15" s="418"/>
       <c r="D15" s="418"/>
@@ -17494,7 +17494,7 @@
       <c r="BU15" s="365"/>
     </row>
     <row r="16" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="1122"/>
+      <c r="A16" s="1127"/>
       <c r="B16" s="385"/>
       <c r="C16" s="386"/>
       <c r="D16" s="386"/>
@@ -17830,108 +17830,108 @@
       <c r="BV19" s="409"/>
     </row>
     <row r="20" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="1120" t="s">
+      <c r="A20" s="1132" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="1116" t="s">
+      <c r="B20" s="1128" t="s">
         <v>39</v>
       </c>
-      <c r="C20" s="1116"/>
-      <c r="D20" s="1116"/>
-      <c r="E20" s="1116"/>
-      <c r="F20" s="1115"/>
+      <c r="C20" s="1128"/>
+      <c r="D20" s="1128"/>
+      <c r="E20" s="1128"/>
+      <c r="F20" s="1129"/>
       <c r="G20" s="838"/>
-      <c r="H20" s="1114" t="s">
+      <c r="H20" s="1130" t="s">
         <v>40</v>
       </c>
-      <c r="I20" s="1114"/>
-      <c r="J20" s="1114"/>
-      <c r="K20" s="1114"/>
-      <c r="L20" s="1114"/>
+      <c r="I20" s="1130"/>
+      <c r="J20" s="1130"/>
+      <c r="K20" s="1130"/>
+      <c r="L20" s="1130"/>
       <c r="M20" s="411"/>
-      <c r="N20" s="1114" t="s">
+      <c r="N20" s="1130" t="s">
         <v>41</v>
       </c>
-      <c r="O20" s="1114"/>
-      <c r="P20" s="1114"/>
-      <c r="Q20" s="1114"/>
-      <c r="R20" s="1114"/>
+      <c r="O20" s="1130"/>
+      <c r="P20" s="1130"/>
+      <c r="Q20" s="1130"/>
+      <c r="R20" s="1130"/>
       <c r="S20" s="838"/>
-      <c r="T20" s="1114" t="s">
+      <c r="T20" s="1130" t="s">
         <v>42</v>
       </c>
-      <c r="U20" s="1114"/>
-      <c r="V20" s="1114"/>
-      <c r="W20" s="1114"/>
-      <c r="X20" s="1114"/>
+      <c r="U20" s="1130"/>
+      <c r="V20" s="1130"/>
+      <c r="W20" s="1130"/>
+      <c r="X20" s="1130"/>
       <c r="Y20" s="411"/>
-      <c r="Z20" s="1116" t="s">
+      <c r="Z20" s="1128" t="s">
         <v>43</v>
       </c>
-      <c r="AA20" s="1116"/>
-      <c r="AB20" s="1116"/>
-      <c r="AC20" s="1116"/>
-      <c r="AD20" s="1116"/>
+      <c r="AA20" s="1128"/>
+      <c r="AB20" s="1128"/>
+      <c r="AC20" s="1128"/>
+      <c r="AD20" s="1128"/>
       <c r="AE20" s="838"/>
-      <c r="AF20" s="1117" t="s">
+      <c r="AF20" s="1133" t="s">
         <v>44</v>
       </c>
-      <c r="AG20" s="1117"/>
-      <c r="AH20" s="1117"/>
-      <c r="AI20" s="1117"/>
-      <c r="AJ20" s="1117"/>
+      <c r="AG20" s="1133"/>
+      <c r="AH20" s="1133"/>
+      <c r="AI20" s="1133"/>
+      <c r="AJ20" s="1133"/>
       <c r="AK20" s="411"/>
-      <c r="AL20" s="1121" t="s">
+      <c r="AL20" s="1134" t="s">
         <v>45</v>
       </c>
-      <c r="AM20" s="1121"/>
-      <c r="AN20" s="1121"/>
-      <c r="AO20" s="1121"/>
-      <c r="AP20" s="1121"/>
+      <c r="AM20" s="1134"/>
+      <c r="AN20" s="1134"/>
+      <c r="AO20" s="1134"/>
+      <c r="AP20" s="1134"/>
       <c r="AQ20" s="838"/>
-      <c r="AR20" s="1114" t="s">
+      <c r="AR20" s="1130" t="s">
         <v>46</v>
       </c>
-      <c r="AS20" s="1114"/>
-      <c r="AT20" s="1114"/>
-      <c r="AU20" s="1114"/>
-      <c r="AV20" s="1114"/>
+      <c r="AS20" s="1130"/>
+      <c r="AT20" s="1130"/>
+      <c r="AU20" s="1130"/>
+      <c r="AV20" s="1130"/>
       <c r="AW20" s="411"/>
-      <c r="AX20" s="1118" t="s">
+      <c r="AX20" s="1131" t="s">
         <v>47</v>
       </c>
-      <c r="AY20" s="1118"/>
-      <c r="AZ20" s="1118"/>
-      <c r="BA20" s="1118"/>
-      <c r="BB20" s="1118"/>
+      <c r="AY20" s="1131"/>
+      <c r="AZ20" s="1131"/>
+      <c r="BA20" s="1131"/>
+      <c r="BB20" s="1131"/>
       <c r="BC20" s="838"/>
-      <c r="BD20" s="1114" t="s">
+      <c r="BD20" s="1130" t="s">
         <v>48</v>
       </c>
-      <c r="BE20" s="1114"/>
-      <c r="BF20" s="1114"/>
-      <c r="BG20" s="1114"/>
-      <c r="BH20" s="1114"/>
+      <c r="BE20" s="1130"/>
+      <c r="BF20" s="1130"/>
+      <c r="BG20" s="1130"/>
+      <c r="BH20" s="1130"/>
       <c r="BI20" s="411"/>
-      <c r="BJ20" s="1115" t="s">
+      <c r="BJ20" s="1129" t="s">
         <v>49</v>
       </c>
-      <c r="BK20" s="1115"/>
-      <c r="BL20" s="1115"/>
-      <c r="BM20" s="1115"/>
-      <c r="BN20" s="1115"/>
+      <c r="BK20" s="1129"/>
+      <c r="BL20" s="1129"/>
+      <c r="BM20" s="1129"/>
+      <c r="BN20" s="1129"/>
       <c r="BO20" s="838"/>
-      <c r="BP20" s="1114" t="s">
+      <c r="BP20" s="1130" t="s">
         <v>50</v>
       </c>
-      <c r="BQ20" s="1114"/>
-      <c r="BR20" s="1114"/>
-      <c r="BS20" s="1114"/>
-      <c r="BT20" s="1114"/>
+      <c r="BQ20" s="1130"/>
+      <c r="BR20" s="1130"/>
+      <c r="BS20" s="1130"/>
+      <c r="BT20" s="1130"/>
       <c r="BU20" s="411"/>
     </row>
     <row r="21" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1120"/>
+      <c r="A21" s="1132"/>
       <c r="B21" s="854" t="s">
         <v>175</v>
       </c>
@@ -18150,7 +18150,7 @@
       </c>
     </row>
     <row r="22" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="1120"/>
+      <c r="A22" s="1132"/>
       <c r="B22" s="412">
         <v>46024</v>
       </c>
@@ -18281,7 +18281,7 @@
       <c r="BU22" s="876"/>
     </row>
     <row r="23" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="1120"/>
+      <c r="A23" s="1132"/>
       <c r="B23" s="378">
         <v>46025</v>
       </c>
@@ -18416,7 +18416,7 @@
       <c r="BU23" s="424"/>
     </row>
     <row r="24" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="1120"/>
+      <c r="A24" s="1132"/>
       <c r="B24" s="378">
         <v>46031</v>
       </c>
@@ -18555,7 +18555,7 @@
       <c r="BU24" s="424"/>
     </row>
     <row r="25" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="1120"/>
+      <c r="A25" s="1132"/>
       <c r="B25" s="378">
         <v>46032</v>
       </c>
@@ -18693,7 +18693,7 @@
       <c r="BU25" s="424"/>
     </row>
     <row r="26" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="1120"/>
+      <c r="A26" s="1132"/>
       <c r="B26" s="930">
         <v>46033</v>
       </c>
@@ -18834,7 +18834,7 @@
       <c r="BU26" s="424"/>
     </row>
     <row r="27" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1120"/>
+      <c r="A27" s="1132"/>
       <c r="B27" s="928">
         <v>46039</v>
       </c>
@@ -18973,7 +18973,7 @@
       <c r="BU27" s="424"/>
     </row>
     <row r="28" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1120"/>
+      <c r="A28" s="1132"/>
       <c r="B28" s="928">
         <v>46040</v>
       </c>
@@ -19112,7 +19112,7 @@
       <c r="BU28" s="424"/>
     </row>
     <row r="29" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="1120"/>
+      <c r="A29" s="1132"/>
       <c r="B29" s="928">
         <v>46041</v>
       </c>
@@ -19253,7 +19253,7 @@
       <c r="BU29" s="424"/>
     </row>
     <row r="30" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="1120"/>
+      <c r="A30" s="1132"/>
       <c r="B30" s="928">
         <v>46042</v>
       </c>
@@ -19392,7 +19392,7 @@
       <c r="BU30" s="424"/>
     </row>
     <row r="31" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="1120"/>
+      <c r="A31" s="1132"/>
       <c r="B31" s="928">
         <v>46050</v>
       </c>
@@ -19527,7 +19527,7 @@
       <c r="BU31" s="424"/>
     </row>
     <row r="32" spans="1:74" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="1120"/>
+      <c r="A32" s="1132"/>
       <c r="B32" s="928"/>
       <c r="C32" s="884"/>
       <c r="D32" s="884"/>
@@ -19662,7 +19662,7 @@
       <c r="BU32" s="424"/>
     </row>
     <row r="33" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1120"/>
+      <c r="A33" s="1132"/>
       <c r="B33" s="928"/>
       <c r="C33" s="884"/>
       <c r="D33" s="884"/>
@@ -19793,7 +19793,7 @@
       <c r="BU33" s="457"/>
     </row>
     <row r="34" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="1120"/>
+      <c r="A34" s="1132"/>
       <c r="B34" s="928"/>
       <c r="C34" s="884"/>
       <c r="D34" s="884"/>
@@ -19922,7 +19922,7 @@
       <c r="BU34" s="424"/>
     </row>
     <row r="35" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1120"/>
+      <c r="A35" s="1132"/>
       <c r="B35" s="928"/>
       <c r="C35" s="884"/>
       <c r="D35" s="884"/>
@@ -20035,7 +20035,7 @@
       <c r="BU35" s="424"/>
     </row>
     <row r="36" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="1120"/>
+      <c r="A36" s="1132"/>
       <c r="B36" s="928"/>
       <c r="C36" s="884"/>
       <c r="D36" s="884"/>
@@ -20148,7 +20148,7 @@
       <c r="BU36" s="424"/>
     </row>
     <row r="37" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="1120"/>
+      <c r="A37" s="1132"/>
       <c r="B37" s="928"/>
       <c r="C37" s="884"/>
       <c r="D37" s="884"/>
@@ -20255,7 +20255,7 @@
       <c r="BU37" s="424"/>
     </row>
     <row r="38" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="1120"/>
+      <c r="A38" s="1132"/>
       <c r="B38" s="928"/>
       <c r="C38" s="884"/>
       <c r="D38" s="884"/>
@@ -20362,7 +20362,7 @@
       <c r="BU38" s="424"/>
     </row>
     <row r="39" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1120"/>
+      <c r="A39" s="1132"/>
       <c r="B39" s="928"/>
       <c r="C39" s="884"/>
       <c r="D39" s="884"/>
@@ -20463,7 +20463,7 @@
       <c r="BU39" s="424"/>
     </row>
     <row r="40" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1120"/>
+      <c r="A40" s="1132"/>
       <c r="B40" s="928"/>
       <c r="C40" s="884"/>
       <c r="D40" s="884"/>
@@ -20554,7 +20554,7 @@
       <c r="BU40" s="424"/>
     </row>
     <row r="41" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1120"/>
+      <c r="A41" s="1132"/>
       <c r="B41" s="928"/>
       <c r="C41" s="884"/>
       <c r="D41" s="884"/>
@@ -20643,7 +20643,7 @@
       <c r="BU41" s="431"/>
     </row>
     <row r="42" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1120"/>
+      <c r="A42" s="1132"/>
       <c r="B42" s="928"/>
       <c r="C42" s="884"/>
       <c r="D42" s="884"/>
@@ -20732,7 +20732,7 @@
       <c r="BU42" s="424"/>
     </row>
     <row r="43" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="1120"/>
+      <c r="A43" s="1132"/>
       <c r="B43" s="928"/>
       <c r="C43" s="884"/>
       <c r="D43" s="884"/>
@@ -20807,7 +20807,7 @@
       <c r="BU43" s="424"/>
     </row>
     <row r="44" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1120"/>
+      <c r="A44" s="1132"/>
       <c r="B44" s="928"/>
       <c r="C44" s="884"/>
       <c r="D44" s="884"/>
@@ -20882,7 +20882,7 @@
       <c r="BU44" s="424"/>
     </row>
     <row r="45" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1120"/>
+      <c r="A45" s="1132"/>
       <c r="B45" s="928"/>
       <c r="C45" s="884"/>
       <c r="D45" s="884"/>
@@ -20957,7 +20957,7 @@
       <c r="BU45" s="424"/>
     </row>
     <row r="46" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1120"/>
+      <c r="A46" s="1132"/>
       <c r="B46" s="928"/>
       <c r="C46" s="884"/>
       <c r="D46" s="884"/>
@@ -21032,7 +21032,7 @@
       <c r="BU46" s="424"/>
     </row>
     <row r="47" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1120"/>
+      <c r="A47" s="1132"/>
       <c r="B47" s="928"/>
       <c r="C47" s="884"/>
       <c r="D47" s="884"/>
@@ -21107,7 +21107,7 @@
       <c r="BU47" s="424"/>
     </row>
     <row r="48" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1120"/>
+      <c r="A48" s="1132"/>
       <c r="B48" s="928"/>
       <c r="C48" s="884"/>
       <c r="D48" s="884"/>
@@ -21182,7 +21182,7 @@
       <c r="BU48" s="424"/>
     </row>
     <row r="49" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1120"/>
+      <c r="A49" s="1132"/>
       <c r="B49" s="928"/>
       <c r="C49" s="884"/>
       <c r="D49" s="884"/>
@@ -21257,7 +21257,7 @@
       <c r="BU49" s="424"/>
     </row>
     <row r="50" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1120"/>
+      <c r="A50" s="1132"/>
       <c r="B50" s="928"/>
       <c r="C50" s="884"/>
       <c r="D50" s="884"/>
@@ -21332,7 +21332,7 @@
       <c r="BU50" s="424"/>
     </row>
     <row r="51" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1120"/>
+      <c r="A51" s="1132"/>
       <c r="B51" s="928"/>
       <c r="C51" s="884"/>
       <c r="D51" s="884"/>
@@ -21407,7 +21407,7 @@
       <c r="BU51" s="424"/>
     </row>
     <row r="52" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1120"/>
+      <c r="A52" s="1132"/>
       <c r="B52" s="401"/>
       <c r="C52" s="397"/>
       <c r="D52" s="886"/>
@@ -21695,108 +21695,108 @@
       <c r="BU55" s="406"/>
     </row>
     <row r="56" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1119" t="s">
+      <c r="A56" s="1135" t="s">
         <v>2</v>
       </c>
-      <c r="B56" s="1115" t="s">
+      <c r="B56" s="1129" t="s">
         <v>39</v>
       </c>
-      <c r="C56" s="1115"/>
-      <c r="D56" s="1115"/>
-      <c r="E56" s="1115"/>
-      <c r="F56" s="1115"/>
+      <c r="C56" s="1129"/>
+      <c r="D56" s="1129"/>
+      <c r="E56" s="1129"/>
+      <c r="F56" s="1129"/>
       <c r="G56" s="838"/>
-      <c r="H56" s="1114" t="s">
+      <c r="H56" s="1130" t="s">
         <v>40</v>
       </c>
-      <c r="I56" s="1114"/>
-      <c r="J56" s="1114"/>
-      <c r="K56" s="1114"/>
-      <c r="L56" s="1114"/>
+      <c r="I56" s="1130"/>
+      <c r="J56" s="1130"/>
+      <c r="K56" s="1130"/>
+      <c r="L56" s="1130"/>
       <c r="M56" s="411"/>
-      <c r="N56" s="1114" t="s">
+      <c r="N56" s="1130" t="s">
         <v>41</v>
       </c>
-      <c r="O56" s="1114"/>
-      <c r="P56" s="1114"/>
-      <c r="Q56" s="1114"/>
-      <c r="R56" s="1114"/>
+      <c r="O56" s="1130"/>
+      <c r="P56" s="1130"/>
+      <c r="Q56" s="1130"/>
+      <c r="R56" s="1130"/>
       <c r="S56" s="838"/>
-      <c r="T56" s="1114" t="s">
+      <c r="T56" s="1130" t="s">
         <v>42</v>
       </c>
-      <c r="U56" s="1114"/>
-      <c r="V56" s="1114"/>
-      <c r="W56" s="1114"/>
-      <c r="X56" s="1114"/>
+      <c r="U56" s="1130"/>
+      <c r="V56" s="1130"/>
+      <c r="W56" s="1130"/>
+      <c r="X56" s="1130"/>
       <c r="Y56" s="411"/>
-      <c r="Z56" s="1116" t="s">
+      <c r="Z56" s="1128" t="s">
         <v>43</v>
       </c>
-      <c r="AA56" s="1116"/>
-      <c r="AB56" s="1116"/>
-      <c r="AC56" s="1116"/>
-      <c r="AD56" s="1116"/>
+      <c r="AA56" s="1128"/>
+      <c r="AB56" s="1128"/>
+      <c r="AC56" s="1128"/>
+      <c r="AD56" s="1128"/>
       <c r="AE56" s="838"/>
-      <c r="AF56" s="1117" t="s">
+      <c r="AF56" s="1133" t="s">
         <v>44</v>
       </c>
-      <c r="AG56" s="1117"/>
-      <c r="AH56" s="1117"/>
-      <c r="AI56" s="1117"/>
-      <c r="AJ56" s="1117"/>
+      <c r="AG56" s="1133"/>
+      <c r="AH56" s="1133"/>
+      <c r="AI56" s="1133"/>
+      <c r="AJ56" s="1133"/>
       <c r="AK56" s="411"/>
-      <c r="AL56" s="1118" t="s">
+      <c r="AL56" s="1131" t="s">
         <v>45</v>
       </c>
-      <c r="AM56" s="1118"/>
-      <c r="AN56" s="1118"/>
-      <c r="AO56" s="1118"/>
-      <c r="AP56" s="1118"/>
+      <c r="AM56" s="1131"/>
+      <c r="AN56" s="1131"/>
+      <c r="AO56" s="1131"/>
+      <c r="AP56" s="1131"/>
       <c r="AQ56" s="838"/>
-      <c r="AR56" s="1114" t="s">
+      <c r="AR56" s="1130" t="s">
         <v>46</v>
       </c>
-      <c r="AS56" s="1114"/>
-      <c r="AT56" s="1114"/>
-      <c r="AU56" s="1114"/>
-      <c r="AV56" s="1114"/>
+      <c r="AS56" s="1130"/>
+      <c r="AT56" s="1130"/>
+      <c r="AU56" s="1130"/>
+      <c r="AV56" s="1130"/>
       <c r="AW56" s="411"/>
-      <c r="AX56" s="1118" t="s">
+      <c r="AX56" s="1131" t="s">
         <v>47</v>
       </c>
-      <c r="AY56" s="1118"/>
-      <c r="AZ56" s="1118"/>
-      <c r="BA56" s="1118"/>
-      <c r="BB56" s="1118"/>
+      <c r="AY56" s="1131"/>
+      <c r="AZ56" s="1131"/>
+      <c r="BA56" s="1131"/>
+      <c r="BB56" s="1131"/>
       <c r="BC56" s="838"/>
-      <c r="BD56" s="1114" t="s">
+      <c r="BD56" s="1130" t="s">
         <v>48</v>
       </c>
-      <c r="BE56" s="1114"/>
-      <c r="BF56" s="1114"/>
-      <c r="BG56" s="1114"/>
-      <c r="BH56" s="1114"/>
+      <c r="BE56" s="1130"/>
+      <c r="BF56" s="1130"/>
+      <c r="BG56" s="1130"/>
+      <c r="BH56" s="1130"/>
       <c r="BI56" s="411"/>
-      <c r="BJ56" s="1115" t="s">
+      <c r="BJ56" s="1129" t="s">
         <v>49</v>
       </c>
-      <c r="BK56" s="1115"/>
-      <c r="BL56" s="1115"/>
-      <c r="BM56" s="1115"/>
-      <c r="BN56" s="1115"/>
+      <c r="BK56" s="1129"/>
+      <c r="BL56" s="1129"/>
+      <c r="BM56" s="1129"/>
+      <c r="BN56" s="1129"/>
       <c r="BO56" s="838"/>
-      <c r="BP56" s="1114" t="s">
+      <c r="BP56" s="1130" t="s">
         <v>50</v>
       </c>
-      <c r="BQ56" s="1114"/>
-      <c r="BR56" s="1114"/>
-      <c r="BS56" s="1114"/>
-      <c r="BT56" s="1114"/>
+      <c r="BQ56" s="1130"/>
+      <c r="BR56" s="1130"/>
+      <c r="BS56" s="1130"/>
+      <c r="BT56" s="1130"/>
       <c r="BU56" s="411"/>
     </row>
     <row r="57" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1119"/>
+      <c r="A57" s="1135"/>
       <c r="B57" s="854" t="s">
         <v>175</v>
       </c>
@@ -22015,7 +22015,7 @@
       </c>
     </row>
     <row r="58" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1119"/>
+      <c r="A58" s="1135"/>
       <c r="B58" s="1042">
         <v>46038</v>
       </c>
@@ -22128,7 +22128,7 @@
       </c>
     </row>
     <row r="59" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1119"/>
+      <c r="A59" s="1135"/>
       <c r="B59" s="378">
         <v>46042</v>
       </c>
@@ -22269,7 +22269,7 @@
       <c r="BU59" s="424"/>
     </row>
     <row r="60" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1119"/>
+      <c r="A60" s="1135"/>
       <c r="B60" s="378">
         <v>46045</v>
       </c>
@@ -22394,7 +22394,7 @@
       <c r="BU60" s="424"/>
     </row>
     <row r="61" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1119"/>
+      <c r="A61" s="1135"/>
       <c r="B61" s="378">
         <v>46045</v>
       </c>
@@ -22519,7 +22519,7 @@
       <c r="BU61" s="424"/>
     </row>
     <row r="62" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1119"/>
+      <c r="A62" s="1135"/>
       <c r="B62" s="378">
         <v>46047</v>
       </c>
@@ -22628,7 +22628,7 @@
       <c r="BU62" s="424"/>
     </row>
     <row r="63" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="1119"/>
+      <c r="A63" s="1135"/>
       <c r="B63" s="378">
         <v>46048</v>
       </c>
@@ -22739,7 +22739,7 @@
       <c r="BU63" s="424"/>
     </row>
     <row r="64" spans="1:73" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1119"/>
+      <c r="A64" s="1135"/>
       <c r="B64" s="378">
         <v>46048</v>
       </c>
@@ -22830,7 +22830,7 @@
       <c r="BU64" s="424"/>
     </row>
     <row r="65" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1119"/>
+      <c r="A65" s="1135"/>
       <c r="B65" s="378">
         <v>46049</v>
       </c>
@@ -22921,7 +22921,7 @@
       <c r="BU65" s="424"/>
     </row>
     <row r="66" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1119"/>
+      <c r="A66" s="1135"/>
       <c r="B66" s="378">
         <v>46049</v>
       </c>
@@ -23014,7 +23014,7 @@
       <c r="BU66" s="424"/>
     </row>
     <row r="67" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="1119"/>
+      <c r="A67" s="1135"/>
       <c r="B67" s="936"/>
       <c r="C67" s="937"/>
       <c r="D67" s="937"/>
@@ -23099,7 +23099,7 @@
       <c r="BU67" s="424"/>
     </row>
     <row r="68" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="1119"/>
+      <c r="A68" s="1135"/>
       <c r="B68" s="474"/>
       <c r="C68" s="373"/>
       <c r="D68" s="373"/>
@@ -23184,7 +23184,7 @@
       <c r="BU68" s="424"/>
     </row>
     <row r="69" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="1119"/>
+      <c r="A69" s="1135"/>
       <c r="B69" s="474"/>
       <c r="C69" s="373"/>
       <c r="D69" s="373"/>
@@ -23267,7 +23267,7 @@
       <c r="BU69" s="424"/>
     </row>
     <row r="70" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1119"/>
+      <c r="A70" s="1135"/>
       <c r="B70" s="474"/>
       <c r="C70" s="373"/>
       <c r="D70" s="373"/>
@@ -23350,7 +23350,7 @@
       <c r="BU70" s="424"/>
     </row>
     <row r="71" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="1119"/>
+      <c r="A71" s="1135"/>
       <c r="B71" s="474"/>
       <c r="C71" s="373"/>
       <c r="D71" s="373"/>
@@ -23425,7 +23425,7 @@
       <c r="BU71" s="424"/>
     </row>
     <row r="72" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="1119"/>
+      <c r="A72" s="1135"/>
       <c r="B72" s="474"/>
       <c r="C72" s="373"/>
       <c r="D72" s="373"/>
@@ -23500,7 +23500,7 @@
       <c r="BU72" s="424"/>
     </row>
     <row r="73" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="1119"/>
+      <c r="A73" s="1135"/>
       <c r="B73" s="474"/>
       <c r="C73" s="373"/>
       <c r="D73" s="373"/>
@@ -23575,7 +23575,7 @@
       <c r="BU73" s="424"/>
     </row>
     <row r="74" spans="1:75" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="1119"/>
+      <c r="A74" s="1135"/>
       <c r="B74" s="464"/>
       <c r="C74" s="397"/>
       <c r="D74" s="397"/>
@@ -29174,16 +29174,19 @@
     </row>
   </sheetData>
   <mergeCells count="39">
-    <mergeCell ref="A1:A16"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="H1:L1"/>
-    <mergeCell ref="N1:R1"/>
-    <mergeCell ref="T1:X1"/>
-    <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="AF1:AJ1"/>
-    <mergeCell ref="AL1:AP1"/>
-    <mergeCell ref="AR1:AV1"/>
-    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="BD56:BH56"/>
+    <mergeCell ref="BJ56:BN56"/>
+    <mergeCell ref="BP56:BT56"/>
+    <mergeCell ref="Z56:AD56"/>
+    <mergeCell ref="AF56:AJ56"/>
+    <mergeCell ref="AL56:AP56"/>
+    <mergeCell ref="AR56:AV56"/>
+    <mergeCell ref="AX56:BB56"/>
+    <mergeCell ref="A56:A74"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="H56:L56"/>
+    <mergeCell ref="N56:R56"/>
+    <mergeCell ref="T56:X56"/>
     <mergeCell ref="BD1:BH1"/>
     <mergeCell ref="BJ1:BN1"/>
     <mergeCell ref="BP1:BT1"/>
@@ -29200,19 +29203,16 @@
     <mergeCell ref="BD20:BH20"/>
     <mergeCell ref="BJ20:BN20"/>
     <mergeCell ref="BP20:BT20"/>
-    <mergeCell ref="A56:A74"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="H56:L56"/>
-    <mergeCell ref="N56:R56"/>
-    <mergeCell ref="T56:X56"/>
-    <mergeCell ref="BD56:BH56"/>
-    <mergeCell ref="BJ56:BN56"/>
-    <mergeCell ref="BP56:BT56"/>
-    <mergeCell ref="Z56:AD56"/>
-    <mergeCell ref="AF56:AJ56"/>
-    <mergeCell ref="AL56:AP56"/>
-    <mergeCell ref="AR56:AV56"/>
-    <mergeCell ref="AX56:BB56"/>
+    <mergeCell ref="Z1:AD1"/>
+    <mergeCell ref="AF1:AJ1"/>
+    <mergeCell ref="AL1:AP1"/>
+    <mergeCell ref="AR1:AV1"/>
+    <mergeCell ref="AX1:BB1"/>
+    <mergeCell ref="A1:A16"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="H1:L1"/>
+    <mergeCell ref="N1:R1"/>
+    <mergeCell ref="T1:X1"/>
   </mergeCells>
   <conditionalFormatting sqref="G78">
     <cfRule type="cellIs" dxfId="30" priority="36" operator="greaterThan">
@@ -29349,100 +29349,100 @@
       <c r="M1" s="525"/>
     </row>
     <row r="2" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H2" s="1133" t="s">
+      <c r="H2" s="1136" t="s">
         <v>509</v>
       </c>
-      <c r="I2" s="1133"/>
-      <c r="J2" s="1133"/>
-      <c r="K2" s="1134" t="s">
+      <c r="I2" s="1136"/>
+      <c r="J2" s="1136"/>
+      <c r="K2" s="1137" t="s">
         <v>510</v>
       </c>
-      <c r="L2" s="1134"/>
-      <c r="M2" s="1134"/>
-      <c r="N2" s="1134" t="s">
+      <c r="L2" s="1137"/>
+      <c r="M2" s="1137"/>
+      <c r="N2" s="1137" t="s">
         <v>192</v>
       </c>
-      <c r="O2" s="1134"/>
-      <c r="P2" s="1134"/>
-      <c r="Q2" s="1134" t="s">
+      <c r="O2" s="1137"/>
+      <c r="P2" s="1137"/>
+      <c r="Q2" s="1137" t="s">
         <v>193</v>
       </c>
-      <c r="R2" s="1134"/>
-      <c r="S2" s="1134"/>
-      <c r="T2" s="1134" t="s">
+      <c r="R2" s="1137"/>
+      <c r="S2" s="1137"/>
+      <c r="T2" s="1137" t="s">
         <v>194</v>
       </c>
-      <c r="U2" s="1134"/>
-      <c r="V2" s="1134"/>
+      <c r="U2" s="1137"/>
+      <c r="V2" s="1137"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H3" s="1133"/>
-      <c r="I3" s="1133"/>
-      <c r="J3" s="1133"/>
-      <c r="K3" s="1134"/>
-      <c r="L3" s="1134"/>
-      <c r="M3" s="1134"/>
-      <c r="N3" s="1134"/>
-      <c r="O3" s="1134"/>
-      <c r="P3" s="1134"/>
-      <c r="Q3" s="1134"/>
-      <c r="R3" s="1134"/>
-      <c r="S3" s="1134"/>
-      <c r="T3" s="1134"/>
-      <c r="U3" s="1134"/>
-      <c r="V3" s="1134"/>
+      <c r="H3" s="1136"/>
+      <c r="I3" s="1136"/>
+      <c r="J3" s="1136"/>
+      <c r="K3" s="1137"/>
+      <c r="L3" s="1137"/>
+      <c r="M3" s="1137"/>
+      <c r="N3" s="1137"/>
+      <c r="O3" s="1137"/>
+      <c r="P3" s="1137"/>
+      <c r="Q3" s="1137"/>
+      <c r="R3" s="1137"/>
+      <c r="S3" s="1137"/>
+      <c r="T3" s="1137"/>
+      <c r="U3" s="1137"/>
+      <c r="V3" s="1137"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H4" s="1133"/>
-      <c r="I4" s="1133"/>
-      <c r="J4" s="1133"/>
-      <c r="K4" s="1134"/>
-      <c r="L4" s="1134"/>
-      <c r="M4" s="1134"/>
-      <c r="N4" s="1134"/>
-      <c r="O4" s="1134"/>
-      <c r="P4" s="1134"/>
-      <c r="Q4" s="1134"/>
-      <c r="R4" s="1134"/>
-      <c r="S4" s="1134"/>
-      <c r="T4" s="1134"/>
-      <c r="U4" s="1134"/>
-      <c r="V4" s="1134"/>
+      <c r="H4" s="1136"/>
+      <c r="I4" s="1136"/>
+      <c r="J4" s="1136"/>
+      <c r="K4" s="1137"/>
+      <c r="L4" s="1137"/>
+      <c r="M4" s="1137"/>
+      <c r="N4" s="1137"/>
+      <c r="O4" s="1137"/>
+      <c r="P4" s="1137"/>
+      <c r="Q4" s="1137"/>
+      <c r="R4" s="1137"/>
+      <c r="S4" s="1137"/>
+      <c r="T4" s="1137"/>
+      <c r="U4" s="1137"/>
+      <c r="V4" s="1137"/>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
-      <c r="H5" s="1133"/>
-      <c r="I5" s="1133"/>
-      <c r="J5" s="1133"/>
-      <c r="K5" s="1134"/>
-      <c r="L5" s="1134"/>
-      <c r="M5" s="1134"/>
-      <c r="N5" s="1134"/>
-      <c r="O5" s="1134"/>
-      <c r="P5" s="1134"/>
-      <c r="Q5" s="1134"/>
-      <c r="R5" s="1134"/>
-      <c r="S5" s="1134"/>
-      <c r="T5" s="1134"/>
-      <c r="U5" s="1134"/>
-      <c r="V5" s="1134"/>
+      <c r="H5" s="1136"/>
+      <c r="I5" s="1136"/>
+      <c r="J5" s="1136"/>
+      <c r="K5" s="1137"/>
+      <c r="L5" s="1137"/>
+      <c r="M5" s="1137"/>
+      <c r="N5" s="1137"/>
+      <c r="O5" s="1137"/>
+      <c r="P5" s="1137"/>
+      <c r="Q5" s="1137"/>
+      <c r="R5" s="1137"/>
+      <c r="S5" s="1137"/>
+      <c r="T5" s="1137"/>
+      <c r="U5" s="1137"/>
+      <c r="V5" s="1137"/>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="G6" s="526"/>
-      <c r="H6" s="1133"/>
-      <c r="I6" s="1133"/>
-      <c r="J6" s="1133"/>
-      <c r="K6" s="1134"/>
-      <c r="L6" s="1134"/>
-      <c r="M6" s="1134"/>
-      <c r="N6" s="1134"/>
-      <c r="O6" s="1134"/>
-      <c r="P6" s="1134"/>
-      <c r="Q6" s="1134"/>
-      <c r="R6" s="1134"/>
-      <c r="S6" s="1134"/>
-      <c r="T6" s="1134"/>
-      <c r="U6" s="1134"/>
-      <c r="V6" s="1134"/>
+      <c r="H6" s="1136"/>
+      <c r="I6" s="1136"/>
+      <c r="J6" s="1136"/>
+      <c r="K6" s="1137"/>
+      <c r="L6" s="1137"/>
+      <c r="M6" s="1137"/>
+      <c r="N6" s="1137"/>
+      <c r="O6" s="1137"/>
+      <c r="P6" s="1137"/>
+      <c r="Q6" s="1137"/>
+      <c r="R6" s="1137"/>
+      <c r="S6" s="1137"/>
+      <c r="T6" s="1137"/>
+      <c r="U6" s="1137"/>
+      <c r="V6" s="1137"/>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="527" t="s">
@@ -36424,8 +36424,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J59 M59">
-    <cfRule type="colorScale" priority="32">
+  <conditionalFormatting sqref="J44 M44">
+    <cfRule type="colorScale" priority="31">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -36436,26 +36436,6 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J60:J78 J41:J43 J80:J104 J45:J58 J106:J126 M60:M78 M41:M43 M80:M104 M45:M58 M106:M126">
     <cfRule type="colorScale" priority="37">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J79 M79">
-    <cfRule type="colorScale" priority="33">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J105 M105">
-    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -36499,8 +36479,28 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M44 J44">
-    <cfRule type="colorScale" priority="31">
+  <conditionalFormatting sqref="M59 J59">
+    <cfRule type="colorScale" priority="32">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M79 J79">
+    <cfRule type="colorScale" priority="33">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M105 J105">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -38303,11 +38303,11 @@
     <row r="35" spans="1:16" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F35" s="610"/>
       <c r="G35" s="610"/>
-      <c r="H35" s="1135" t="s">
+      <c r="H35" s="1114" t="s">
         <v>272</v>
       </c>
-      <c r="I35" s="1136"/>
-      <c r="J35" s="1137"/>
+      <c r="I35" s="1115"/>
+      <c r="J35" s="1116"/>
       <c r="K35" s="643" t="s">
         <v>273</v>
       </c>
@@ -38733,31 +38733,31 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="1146" t="s">
+      <c r="B1" s="1140" t="s">
         <v>287</v>
       </c>
-      <c r="C1" s="1139" t="s">
+      <c r="C1" s="1141" t="s">
         <v>288</v>
       </c>
-      <c r="D1" s="1157" t="s">
+      <c r="D1" s="1149" t="s">
         <v>67</v>
       </c>
-      <c r="E1" s="1158"/>
-      <c r="F1" s="1158"/>
-      <c r="G1" s="1158"/>
-      <c r="H1" s="1159"/>
-      <c r="I1" s="1154" t="s">
+      <c r="E1" s="1150"/>
+      <c r="F1" s="1150"/>
+      <c r="G1" s="1150"/>
+      <c r="H1" s="1151"/>
+      <c r="I1" s="1142" t="s">
         <v>286</v>
       </c>
-      <c r="J1" s="1147"/>
+      <c r="J1" s="1143"/>
     </row>
     <row r="2" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="1146"/>
-      <c r="C2" s="1139"/>
-      <c r="D2" s="1155" t="s">
+      <c r="B2" s="1140"/>
+      <c r="C2" s="1141"/>
+      <c r="D2" s="1144" t="s">
         <v>289</v>
       </c>
-      <c r="E2" s="1156"/>
+      <c r="E2" s="1145"/>
       <c r="F2" s="1023" t="s">
         <v>291</v>
       </c>
@@ -38767,12 +38767,12 @@
       <c r="H2" s="1081" t="s">
         <v>291</v>
       </c>
-      <c r="I2" s="1154"/>
-      <c r="J2" s="1147"/>
+      <c r="I2" s="1142"/>
+      <c r="J2" s="1143"/>
     </row>
     <row r="3" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1146"/>
-      <c r="C3" s="1139"/>
+      <c r="B3" s="1140"/>
+      <c r="C3" s="1141"/>
       <c r="D3" s="1107"/>
       <c r="E3" s="1016"/>
       <c r="F3" s="1017"/>
@@ -38790,10 +38790,10 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="1140">
-        <v>0</v>
-      </c>
-      <c r="B4" s="1142">
+      <c r="A4" s="1157">
+        <v>0</v>
+      </c>
+      <c r="B4" s="1146">
         <v>2022</v>
       </c>
       <c r="C4" s="687">
@@ -38815,8 +38815,8 @@
       <c r="L4" s="662"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="1143"/>
-      <c r="B5" s="1145"/>
+      <c r="A5" s="1158"/>
+      <c r="B5" s="1147"/>
       <c r="C5" s="664">
         <v>2</v>
       </c>
@@ -38836,8 +38836,8 @@
       <c r="L5" s="670"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="1143"/>
-      <c r="B6" s="1145"/>
+      <c r="A6" s="1158"/>
+      <c r="B6" s="1147"/>
       <c r="C6" s="664">
         <v>3</v>
       </c>
@@ -38857,8 +38857,8 @@
       <c r="L6" s="670"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="1143"/>
-      <c r="B7" s="1145"/>
+      <c r="A7" s="1158"/>
+      <c r="B7" s="1147"/>
       <c r="C7" s="664">
         <v>4</v>
       </c>
@@ -38878,8 +38878,8 @@
       <c r="L7" s="670"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="1143"/>
-      <c r="B8" s="1145"/>
+      <c r="A8" s="1158"/>
+      <c r="B8" s="1147"/>
       <c r="C8" s="664">
         <v>5</v>
       </c>
@@ -38899,8 +38899,8 @@
       <c r="L8" s="670"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="1143"/>
-      <c r="B9" s="1145"/>
+      <c r="A9" s="1158"/>
+      <c r="B9" s="1147"/>
       <c r="C9" s="664">
         <v>6</v>
       </c>
@@ -38920,8 +38920,8 @@
       <c r="L9" s="670"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="1143"/>
-      <c r="B10" s="1145"/>
+      <c r="A10" s="1158"/>
+      <c r="B10" s="1147"/>
       <c r="C10" s="664">
         <v>7</v>
       </c>
@@ -38941,8 +38941,8 @@
       <c r="L10" s="670"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="1143"/>
-      <c r="B11" s="1145"/>
+      <c r="A11" s="1158"/>
+      <c r="B11" s="1147"/>
       <c r="C11" s="664">
         <v>8</v>
       </c>
@@ -38962,8 +38962,8 @@
       <c r="L11" s="681"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="1143"/>
-      <c r="B12" s="1145"/>
+      <c r="A12" s="1158"/>
+      <c r="B12" s="1147"/>
       <c r="C12" s="664">
         <v>9</v>
       </c>
@@ -38983,8 +38983,8 @@
       <c r="L12" s="681"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="1143"/>
-      <c r="B13" s="1145"/>
+      <c r="A13" s="1158"/>
+      <c r="B13" s="1147"/>
       <c r="C13" s="664">
         <v>10</v>
       </c>
@@ -39004,8 +39004,8 @@
       <c r="L13" s="681"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="1143"/>
-      <c r="B14" s="1145"/>
+      <c r="A14" s="1158"/>
+      <c r="B14" s="1147"/>
       <c r="C14" s="664">
         <v>11</v>
       </c>
@@ -39025,8 +39025,8 @@
       <c r="L14" s="681"/>
     </row>
     <row r="15" spans="1:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="1144"/>
-      <c r="B15" s="1141"/>
+      <c r="A15" s="1159"/>
+      <c r="B15" s="1148"/>
       <c r="C15" s="693">
         <v>12</v>
       </c>
@@ -39046,10 +39046,10 @@
       <c r="L15" s="697"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="1140">
-        <v>0</v>
-      </c>
-      <c r="B16" s="1142">
+      <c r="A16" s="1157">
+        <v>0</v>
+      </c>
+      <c r="B16" s="1146">
         <v>2023</v>
       </c>
       <c r="C16" s="687">
@@ -39071,8 +39071,8 @@
       <c r="L16" s="662"/>
     </row>
     <row r="17" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A17" s="1143"/>
-      <c r="B17" s="1145"/>
+      <c r="A17" s="1158"/>
+      <c r="B17" s="1147"/>
       <c r="C17" s="664">
         <v>2</v>
       </c>
@@ -39092,8 +39092,8 @@
       <c r="L17" s="670"/>
     </row>
     <row r="18" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A18" s="1143"/>
-      <c r="B18" s="1145"/>
+      <c r="A18" s="1158"/>
+      <c r="B18" s="1147"/>
       <c r="C18" s="664">
         <v>3</v>
       </c>
@@ -39113,8 +39113,8 @@
       <c r="L18" s="670"/>
     </row>
     <row r="19" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A19" s="1143"/>
-      <c r="B19" s="1145"/>
+      <c r="A19" s="1158"/>
+      <c r="B19" s="1147"/>
       <c r="C19" s="664">
         <v>4</v>
       </c>
@@ -39134,8 +39134,8 @@
       <c r="L19" s="670"/>
     </row>
     <row r="20" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A20" s="1143"/>
-      <c r="B20" s="1145"/>
+      <c r="A20" s="1158"/>
+      <c r="B20" s="1147"/>
       <c r="C20" s="664">
         <v>5</v>
       </c>
@@ -39155,8 +39155,8 @@
       <c r="L20" s="670"/>
     </row>
     <row r="21" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A21" s="1143"/>
-      <c r="B21" s="1145"/>
+      <c r="A21" s="1158"/>
+      <c r="B21" s="1147"/>
       <c r="C21" s="664">
         <v>6</v>
       </c>
@@ -39176,8 +39176,8 @@
       <c r="L21" s="670"/>
     </row>
     <row r="22" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A22" s="1143"/>
-      <c r="B22" s="1145"/>
+      <c r="A22" s="1158"/>
+      <c r="B22" s="1147"/>
       <c r="C22" s="664">
         <v>7</v>
       </c>
@@ -39197,8 +39197,8 @@
       <c r="L22" s="670"/>
     </row>
     <row r="23" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A23" s="1143"/>
-      <c r="B23" s="1145"/>
+      <c r="A23" s="1158"/>
+      <c r="B23" s="1147"/>
       <c r="C23" s="664">
         <v>8</v>
       </c>
@@ -39218,8 +39218,8 @@
       <c r="L23" s="681"/>
     </row>
     <row r="24" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A24" s="1143"/>
-      <c r="B24" s="1145"/>
+      <c r="A24" s="1158"/>
+      <c r="B24" s="1147"/>
       <c r="C24" s="664">
         <v>9</v>
       </c>
@@ -39239,8 +39239,8 @@
       <c r="L24" s="681"/>
     </row>
     <row r="25" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A25" s="1143"/>
-      <c r="B25" s="1145"/>
+      <c r="A25" s="1158"/>
+      <c r="B25" s="1147"/>
       <c r="C25" s="664">
         <v>10</v>
       </c>
@@ -39260,8 +39260,8 @@
       <c r="L25" s="681"/>
     </row>
     <row r="26" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A26" s="1143"/>
-      <c r="B26" s="1145"/>
+      <c r="A26" s="1158"/>
+      <c r="B26" s="1147"/>
       <c r="C26" s="664">
         <v>11</v>
       </c>
@@ -39281,8 +39281,8 @@
       <c r="L26" s="681"/>
     </row>
     <row r="27" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1144"/>
-      <c r="B27" s="1141"/>
+      <c r="A27" s="1159"/>
+      <c r="B27" s="1148"/>
       <c r="C27" s="693">
         <v>12</v>
       </c>
@@ -39302,10 +39302,10 @@
       <c r="L27" s="697"/>
     </row>
     <row r="28" spans="1:46" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="1140">
+      <c r="A28" s="1157">
         <v>1</v>
       </c>
-      <c r="B28" s="1142">
+      <c r="B28" s="1146">
         <v>2024</v>
       </c>
       <c r="C28" s="687">
@@ -39328,46 +39328,46 @@
       <c r="M28" s="663"/>
       <c r="N28" s="663"/>
       <c r="O28" s="663"/>
-      <c r="P28" s="1152" t="s">
+      <c r="P28" s="1138" t="s">
         <v>294</v>
       </c>
-      <c r="Q28" s="1152"/>
-      <c r="R28" s="1152"/>
-      <c r="S28" s="1152"/>
-      <c r="T28" s="1152"/>
-      <c r="U28" s="1152"/>
-      <c r="V28" s="1152"/>
-      <c r="X28" s="1152" t="s">
+      <c r="Q28" s="1138"/>
+      <c r="R28" s="1138"/>
+      <c r="S28" s="1138"/>
+      <c r="T28" s="1138"/>
+      <c r="U28" s="1138"/>
+      <c r="V28" s="1138"/>
+      <c r="X28" s="1138" t="s">
         <v>295</v>
       </c>
-      <c r="Y28" s="1152"/>
-      <c r="Z28" s="1152"/>
-      <c r="AA28" s="1152"/>
-      <c r="AB28" s="1152"/>
-      <c r="AC28" s="1152"/>
-      <c r="AD28" s="1152"/>
-      <c r="AF28" s="1153" t="s">
+      <c r="Y28" s="1138"/>
+      <c r="Z28" s="1138"/>
+      <c r="AA28" s="1138"/>
+      <c r="AB28" s="1138"/>
+      <c r="AC28" s="1138"/>
+      <c r="AD28" s="1138"/>
+      <c r="AF28" s="1139" t="s">
         <v>296</v>
       </c>
-      <c r="AG28" s="1153"/>
-      <c r="AH28" s="1153"/>
-      <c r="AI28" s="1153"/>
-      <c r="AJ28" s="1153"/>
-      <c r="AK28" s="1153"/>
-      <c r="AL28" s="1153"/>
-      <c r="AN28" s="1153" t="s">
+      <c r="AG28" s="1139"/>
+      <c r="AH28" s="1139"/>
+      <c r="AI28" s="1139"/>
+      <c r="AJ28" s="1139"/>
+      <c r="AK28" s="1139"/>
+      <c r="AL28" s="1139"/>
+      <c r="AN28" s="1139" t="s">
         <v>297</v>
       </c>
-      <c r="AO28" s="1153"/>
-      <c r="AP28" s="1153"/>
-      <c r="AQ28" s="1153"/>
-      <c r="AR28" s="1153"/>
-      <c r="AS28" s="1153"/>
-      <c r="AT28" s="1153"/>
+      <c r="AO28" s="1139"/>
+      <c r="AP28" s="1139"/>
+      <c r="AQ28" s="1139"/>
+      <c r="AR28" s="1139"/>
+      <c r="AS28" s="1139"/>
+      <c r="AT28" s="1139"/>
     </row>
     <row r="29" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A29" s="1143"/>
-      <c r="B29" s="1145"/>
+      <c r="A29" s="1158"/>
+      <c r="B29" s="1147"/>
       <c r="C29" s="664">
         <v>2</v>
       </c>
@@ -39441,8 +39441,8 @@
       </c>
     </row>
     <row r="30" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A30" s="1143"/>
-      <c r="B30" s="1145"/>
+      <c r="A30" s="1158"/>
+      <c r="B30" s="1147"/>
       <c r="C30" s="664">
         <v>3</v>
       </c>
@@ -39516,8 +39516,8 @@
       <c r="AT30" s="676"/>
     </row>
     <row r="31" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A31" s="1143"/>
-      <c r="B31" s="1145"/>
+      <c r="A31" s="1158"/>
+      <c r="B31" s="1147"/>
       <c r="C31" s="664">
         <v>4</v>
       </c>
@@ -39555,8 +39555,8 @@
       <c r="AT31" s="676"/>
     </row>
     <row r="32" spans="1:46" x14ac:dyDescent="0.2">
-      <c r="A32" s="1143"/>
-      <c r="B32" s="1145"/>
+      <c r="A32" s="1158"/>
+      <c r="B32" s="1147"/>
       <c r="C32" s="664">
         <v>5</v>
       </c>
@@ -39626,8 +39626,8 @@
       <c r="AT32" s="676"/>
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A33" s="1143"/>
-      <c r="B33" s="1145"/>
+      <c r="A33" s="1158"/>
+      <c r="B33" s="1147"/>
       <c r="C33" s="664">
         <v>6</v>
       </c>
@@ -39695,8 +39695,8 @@
       <c r="AT33" s="676"/>
     </row>
     <row r="34" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A34" s="1143"/>
-      <c r="B34" s="1145"/>
+      <c r="A34" s="1158"/>
+      <c r="B34" s="1147"/>
       <c r="C34" s="664">
         <v>7</v>
       </c>
@@ -39758,8 +39758,8 @@
       <c r="AT34" s="676"/>
     </row>
     <row r="35" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A35" s="1143"/>
-      <c r="B35" s="1145"/>
+      <c r="A35" s="1158"/>
+      <c r="B35" s="1147"/>
       <c r="C35" s="664">
         <v>8</v>
       </c>
@@ -39829,8 +39829,8 @@
       </c>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A36" s="1143"/>
-      <c r="B36" s="1145"/>
+      <c r="A36" s="1158"/>
+      <c r="B36" s="1147"/>
       <c r="C36" s="664">
         <v>9</v>
       </c>
@@ -39896,8 +39896,8 @@
       <c r="AT36" s="676"/>
     </row>
     <row r="37" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A37" s="1143"/>
-      <c r="B37" s="1145"/>
+      <c r="A37" s="1158"/>
+      <c r="B37" s="1147"/>
       <c r="C37" s="664">
         <v>10</v>
       </c>
@@ -39991,8 +39991,8 @@
       </c>
     </row>
     <row r="38" spans="1:47" x14ac:dyDescent="0.2">
-      <c r="A38" s="1143"/>
-      <c r="B38" s="1145"/>
+      <c r="A38" s="1158"/>
+      <c r="B38" s="1147"/>
       <c r="C38" s="664">
         <v>11</v>
       </c>
@@ -40030,8 +40030,8 @@
       <c r="AT38" s="676"/>
     </row>
     <row r="39" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="1144"/>
-      <c r="B39" s="1141"/>
+      <c r="A39" s="1159"/>
+      <c r="B39" s="1148"/>
       <c r="C39" s="693">
         <v>12</v>
       </c>
@@ -40108,10 +40108,10 @@
       </c>
     </row>
     <row r="40" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="1138">
+      <c r="A40" s="1156">
         <v>2</v>
       </c>
-      <c r="B40" s="1139">
+      <c r="B40" s="1141">
         <v>2025</v>
       </c>
       <c r="C40" s="687">
@@ -40184,8 +40184,8 @@
       <c r="AT40" s="676"/>
     </row>
     <row r="41" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="1138"/>
-      <c r="B41" s="1139"/>
+      <c r="A41" s="1156"/>
+      <c r="B41" s="1141"/>
       <c r="C41" s="664">
         <v>2</v>
       </c>
@@ -40247,8 +40247,8 @@
       <c r="AT41" s="676"/>
     </row>
     <row r="42" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="1138"/>
-      <c r="B42" s="1139"/>
+      <c r="A42" s="1156"/>
+      <c r="B42" s="1141"/>
       <c r="C42" s="664">
         <v>3</v>
       </c>
@@ -40318,8 +40318,8 @@
       </c>
     </row>
     <row r="43" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="1138"/>
-      <c r="B43" s="1139"/>
+      <c r="A43" s="1156"/>
+      <c r="B43" s="1141"/>
       <c r="C43" s="664">
         <v>4</v>
       </c>
@@ -40385,8 +40385,8 @@
       <c r="AT43" s="676"/>
     </row>
     <row r="44" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="1138"/>
-      <c r="B44" s="1139"/>
+      <c r="A44" s="1156"/>
+      <c r="B44" s="1141"/>
       <c r="C44" s="664">
         <v>5</v>
       </c>
@@ -40480,8 +40480,8 @@
       </c>
     </row>
     <row r="45" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1138"/>
-      <c r="B45" s="1139"/>
+      <c r="A45" s="1156"/>
+      <c r="B45" s="1141"/>
       <c r="C45" s="664">
         <v>6</v>
       </c>
@@ -40519,8 +40519,8 @@
       <c r="AT45" s="676"/>
     </row>
     <row r="46" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="1138"/>
-      <c r="B46" s="1139"/>
+      <c r="A46" s="1156"/>
+      <c r="B46" s="1141"/>
       <c r="C46" s="664">
         <v>7</v>
       </c>
@@ -40597,8 +40597,8 @@
       </c>
     </row>
     <row r="47" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="1138"/>
-      <c r="B47" s="1139"/>
+      <c r="A47" s="1156"/>
+      <c r="B47" s="1141"/>
       <c r="C47" s="664">
         <v>8</v>
       </c>
@@ -40667,8 +40667,8 @@
       <c r="AT47" s="676"/>
     </row>
     <row r="48" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="1138"/>
-      <c r="B48" s="1139"/>
+      <c r="A48" s="1156"/>
+      <c r="B48" s="1141"/>
       <c r="C48" s="664">
         <v>9</v>
       </c>
@@ -40730,8 +40730,8 @@
       <c r="AT48" s="676"/>
     </row>
     <row r="49" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="1138"/>
-      <c r="B49" s="1139"/>
+      <c r="A49" s="1156"/>
+      <c r="B49" s="1141"/>
       <c r="C49" s="664">
         <v>10</v>
       </c>
@@ -40801,8 +40801,8 @@
       </c>
     </row>
     <row r="50" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="1138"/>
-      <c r="B50" s="1139"/>
+      <c r="A50" s="1156"/>
+      <c r="B50" s="1141"/>
       <c r="C50" s="664">
         <v>11</v>
       </c>
@@ -40874,8 +40874,8 @@
       <c r="AT50" s="676"/>
     </row>
     <row r="51" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="1138"/>
-      <c r="B51" s="1139"/>
+      <c r="A51" s="1156"/>
+      <c r="B51" s="1141"/>
       <c r="C51" s="693">
         <v>12</v>
       </c>
@@ -40969,10 +40969,10 @@
       </c>
     </row>
     <row r="52" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="1138">
+      <c r="A52" s="1156">
         <v>3</v>
       </c>
-      <c r="B52" s="1139">
+      <c r="B52" s="1141">
         <v>2026</v>
       </c>
       <c r="C52" s="687">
@@ -41012,8 +41012,8 @@
       <c r="AT52" s="676"/>
     </row>
     <row r="53" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="1138"/>
-      <c r="B53" s="1139"/>
+      <c r="A53" s="1156"/>
+      <c r="B53" s="1141"/>
       <c r="C53" s="664">
         <v>2</v>
       </c>
@@ -41090,8 +41090,8 @@
       </c>
     </row>
     <row r="54" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="1138"/>
-      <c r="B54" s="1139"/>
+      <c r="A54" s="1156"/>
+      <c r="B54" s="1141"/>
       <c r="C54" s="664">
         <v>3</v>
       </c>
@@ -41160,8 +41160,8 @@
       <c r="AT54" s="676"/>
     </row>
     <row r="55" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="1138"/>
-      <c r="B55" s="1139"/>
+      <c r="A55" s="1156"/>
+      <c r="B55" s="1141"/>
       <c r="C55" s="664">
         <v>4</v>
       </c>
@@ -41232,8 +41232,8 @@
       <c r="AT55" s="676"/>
     </row>
     <row r="56" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="1138"/>
-      <c r="B56" s="1139"/>
+      <c r="A56" s="1156"/>
+      <c r="B56" s="1141"/>
       <c r="C56" s="664">
         <v>5</v>
       </c>
@@ -41306,8 +41306,8 @@
       </c>
     </row>
     <row r="57" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="1138"/>
-      <c r="B57" s="1139"/>
+      <c r="A57" s="1156"/>
+      <c r="B57" s="1141"/>
       <c r="C57" s="664">
         <v>6</v>
       </c>
@@ -41385,8 +41385,8 @@
       <c r="AT57" s="676"/>
     </row>
     <row r="58" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="1138"/>
-      <c r="B58" s="1139"/>
+      <c r="A58" s="1156"/>
+      <c r="B58" s="1141"/>
       <c r="C58" s="664">
         <v>7</v>
       </c>
@@ -41487,8 +41487,8 @@
       </c>
     </row>
     <row r="59" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="1138"/>
-      <c r="B59" s="1139"/>
+      <c r="A59" s="1156"/>
+      <c r="B59" s="1141"/>
       <c r="C59" s="664">
         <v>8</v>
       </c>
@@ -41529,30 +41529,30 @@
       <c r="AT59" s="676"/>
     </row>
     <row r="60" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="1138"/>
-      <c r="B60" s="1139"/>
+      <c r="A60" s="1156"/>
+      <c r="B60" s="1141"/>
       <c r="C60" s="664">
         <v>9</v>
       </c>
       <c r="D60" s="1067"/>
-      <c r="E60" s="667">
+      <c r="E60" s="976">
         <v>720.2</v>
       </c>
-      <c r="F60" s="1077">
+      <c r="F60" s="1076">
         <f t="shared" si="3"/>
         <v>35754.730000000003</v>
       </c>
-      <c r="G60" s="1098">
+      <c r="G60" s="1092">
         <v>82.59</v>
       </c>
-      <c r="H60" s="1099">
+      <c r="H60" s="1095">
         <f>SUM(G60:$G$107)</f>
         <v>2059.1799999999994</v>
       </c>
-      <c r="I60" s="1058">
+      <c r="I60" s="1055">
         <v>500</v>
       </c>
-      <c r="J60" s="679">
+      <c r="J60" s="668">
         <f t="shared" si="2"/>
         <v>19500</v>
       </c>
@@ -41614,8 +41614,8 @@
       </c>
     </row>
     <row r="61" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="1138"/>
-      <c r="B61" s="1139"/>
+      <c r="A61" s="1156"/>
+      <c r="B61" s="1141"/>
       <c r="C61" s="664">
         <v>10</v>
       </c>
@@ -41687,8 +41687,8 @@
       <c r="AT61" s="676"/>
     </row>
     <row r="62" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="1138"/>
-      <c r="B62" s="1139"/>
+      <c r="A62" s="1156"/>
+      <c r="B62" s="1141"/>
       <c r="C62" s="664">
         <v>11</v>
       </c>
@@ -41757,8 +41757,8 @@
       <c r="AT62" s="676"/>
     </row>
     <row r="63" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="1138"/>
-      <c r="B63" s="1139"/>
+      <c r="A63" s="1156"/>
+      <c r="B63" s="1141"/>
       <c r="C63" s="693">
         <v>12</v>
       </c>
@@ -41841,10 +41841,10 @@
       </c>
     </row>
     <row r="64" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="1138">
+      <c r="A64" s="1156">
         <v>4</v>
       </c>
-      <c r="B64" s="1139">
+      <c r="B64" s="1141">
         <v>2027</v>
       </c>
       <c r="C64" s="687">
@@ -41925,8 +41925,8 @@
       <c r="AT64" s="676"/>
     </row>
     <row r="65" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="1138"/>
-      <c r="B65" s="1139"/>
+      <c r="A65" s="1156"/>
+      <c r="B65" s="1141"/>
       <c r="C65" s="664">
         <v>2</v>
       </c>
@@ -42031,8 +42031,8 @@
       </c>
     </row>
     <row r="66" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1138"/>
-      <c r="B66" s="1139"/>
+      <c r="A66" s="1156"/>
+      <c r="B66" s="1141"/>
       <c r="C66" s="664">
         <v>3</v>
       </c>
@@ -42071,8 +42071,8 @@
       <c r="AT66" s="676"/>
     </row>
     <row r="67" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="1138"/>
-      <c r="B67" s="1139"/>
+      <c r="A67" s="1156"/>
+      <c r="B67" s="1141"/>
       <c r="C67" s="664">
         <v>4</v>
       </c>
@@ -42123,8 +42123,8 @@
       </c>
     </row>
     <row r="68" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="1138"/>
-      <c r="B68" s="1139"/>
+      <c r="A68" s="1156"/>
+      <c r="B68" s="1141"/>
       <c r="C68" s="664">
         <v>5</v>
       </c>
@@ -42166,8 +42166,8 @@
       <c r="AT68" s="676"/>
     </row>
     <row r="69" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="1138"/>
-      <c r="B69" s="1139"/>
+      <c r="A69" s="1156"/>
+      <c r="B69" s="1141"/>
       <c r="C69" s="664">
         <v>6</v>
       </c>
@@ -42209,8 +42209,8 @@
       <c r="AT69" s="676"/>
     </row>
     <row r="70" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="1138"/>
-      <c r="B70" s="1139"/>
+      <c r="A70" s="1156"/>
+      <c r="B70" s="1141"/>
       <c r="C70" s="664">
         <v>7</v>
       </c>
@@ -42254,8 +42254,8 @@
       </c>
     </row>
     <row r="71" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="1138"/>
-      <c r="B71" s="1139"/>
+      <c r="A71" s="1156"/>
+      <c r="B71" s="1141"/>
       <c r="C71" s="664">
         <v>8</v>
       </c>
@@ -42301,8 +42301,8 @@
       <c r="AT71" s="676"/>
     </row>
     <row r="72" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="1138"/>
-      <c r="B72" s="1139"/>
+      <c r="A72" s="1156"/>
+      <c r="B72" s="1141"/>
       <c r="C72" s="664">
         <v>9</v>
       </c>
@@ -42354,8 +42354,8 @@
       </c>
     </row>
     <row r="73" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="1138"/>
-      <c r="B73" s="1139"/>
+      <c r="A73" s="1156"/>
+      <c r="B73" s="1141"/>
       <c r="C73" s="664">
         <v>10</v>
       </c>
@@ -42396,8 +42396,8 @@
       </c>
     </row>
     <row r="74" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="1138"/>
-      <c r="B74" s="1139"/>
+      <c r="A74" s="1156"/>
+      <c r="B74" s="1141"/>
       <c r="C74" s="664">
         <v>11</v>
       </c>
@@ -42437,8 +42437,8 @@
       </c>
     </row>
     <row r="75" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="1138"/>
-      <c r="B75" s="1139"/>
+      <c r="A75" s="1156"/>
+      <c r="B75" s="1141"/>
       <c r="C75" s="693">
         <v>12</v>
       </c>
@@ -42486,10 +42486,10 @@
       </c>
     </row>
     <row r="76" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="1138">
+      <c r="A76" s="1156">
         <v>5</v>
       </c>
-      <c r="B76" s="1139">
+      <c r="B76" s="1141">
         <v>2028</v>
       </c>
       <c r="C76" s="687">
@@ -42528,8 +42528,8 @@
       </c>
     </row>
     <row r="77" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="1138"/>
-      <c r="B77" s="1139"/>
+      <c r="A77" s="1156"/>
+      <c r="B77" s="1141"/>
       <c r="C77" s="664">
         <v>2</v>
       </c>
@@ -42566,8 +42566,8 @@
       </c>
     </row>
     <row r="78" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1138"/>
-      <c r="B78" s="1139"/>
+      <c r="A78" s="1156"/>
+      <c r="B78" s="1141"/>
       <c r="C78" s="664">
         <v>3</v>
       </c>
@@ -42604,8 +42604,8 @@
       </c>
     </row>
     <row r="79" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="1138"/>
-      <c r="B79" s="1139"/>
+      <c r="A79" s="1156"/>
+      <c r="B79" s="1141"/>
       <c r="C79" s="664">
         <v>4</v>
       </c>
@@ -42639,8 +42639,8 @@
       </c>
     </row>
     <row r="80" spans="1:47" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="1138"/>
-      <c r="B80" s="1139"/>
+      <c r="A80" s="1156"/>
+      <c r="B80" s="1141"/>
       <c r="C80" s="664">
         <v>5</v>
       </c>
@@ -42677,8 +42677,8 @@
       </c>
     </row>
     <row r="81" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="1138"/>
-      <c r="B81" s="1139"/>
+      <c r="A81" s="1156"/>
+      <c r="B81" s="1141"/>
       <c r="C81" s="664">
         <v>6</v>
       </c>
@@ -42715,8 +42715,8 @@
       </c>
     </row>
     <row r="82" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="1138"/>
-      <c r="B82" s="1139"/>
+      <c r="A82" s="1156"/>
+      <c r="B82" s="1141"/>
       <c r="C82" s="664">
         <v>7</v>
       </c>
@@ -42753,8 +42753,8 @@
       </c>
     </row>
     <row r="83" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="1138"/>
-      <c r="B83" s="1139"/>
+      <c r="A83" s="1156"/>
+      <c r="B83" s="1141"/>
       <c r="C83" s="664">
         <v>8</v>
       </c>
@@ -42788,8 +42788,8 @@
       </c>
     </row>
     <row r="84" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="1138"/>
-      <c r="B84" s="1139"/>
+      <c r="A84" s="1156"/>
+      <c r="B84" s="1141"/>
       <c r="C84" s="664">
         <v>9</v>
       </c>
@@ -42823,8 +42823,8 @@
       </c>
     </row>
     <row r="85" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="1138"/>
-      <c r="B85" s="1139"/>
+      <c r="A85" s="1156"/>
+      <c r="B85" s="1141"/>
       <c r="C85" s="664">
         <v>10</v>
       </c>
@@ -42858,8 +42858,8 @@
       </c>
     </row>
     <row r="86" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="1138"/>
-      <c r="B86" s="1139"/>
+      <c r="A86" s="1156"/>
+      <c r="B86" s="1141"/>
       <c r="C86" s="664">
         <v>11</v>
       </c>
@@ -42893,8 +42893,8 @@
       </c>
     </row>
     <row r="87" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="1138"/>
-      <c r="B87" s="1139"/>
+      <c r="A87" s="1156"/>
+      <c r="B87" s="1141"/>
       <c r="C87" s="693">
         <v>12</v>
       </c>
@@ -42932,10 +42932,10 @@
       </c>
     </row>
     <row r="88" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="1138">
+      <c r="A88" s="1156">
         <v>6</v>
       </c>
-      <c r="B88" s="1139">
+      <c r="B88" s="1141">
         <v>2029</v>
       </c>
       <c r="C88" s="687">
@@ -42971,8 +42971,8 @@
       </c>
     </row>
     <row r="89" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="1138"/>
-      <c r="B89" s="1139"/>
+      <c r="A89" s="1156"/>
+      <c r="B89" s="1141"/>
       <c r="C89" s="664">
         <v>2</v>
       </c>
@@ -43006,8 +43006,8 @@
       </c>
     </row>
     <row r="90" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="1138"/>
-      <c r="B90" s="1139"/>
+      <c r="A90" s="1156"/>
+      <c r="B90" s="1141"/>
       <c r="C90" s="664">
         <v>3</v>
       </c>
@@ -43041,8 +43041,8 @@
       </c>
     </row>
     <row r="91" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="1138"/>
-      <c r="B91" s="1139"/>
+      <c r="A91" s="1156"/>
+      <c r="B91" s="1141"/>
       <c r="C91" s="664">
         <v>4</v>
       </c>
@@ -43077,8 +43077,8 @@
       <c r="M91" s="686"/>
     </row>
     <row r="92" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="1138"/>
-      <c r="B92" s="1139"/>
+      <c r="A92" s="1156"/>
+      <c r="B92" s="1141"/>
       <c r="C92" s="664">
         <v>5</v>
       </c>
@@ -43112,8 +43112,8 @@
       </c>
     </row>
     <row r="93" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="1138"/>
-      <c r="B93" s="1139"/>
+      <c r="A93" s="1156"/>
+      <c r="B93" s="1141"/>
       <c r="C93" s="664">
         <v>6</v>
       </c>
@@ -43148,8 +43148,8 @@
       <c r="M93" s="686"/>
     </row>
     <row r="94" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="1138"/>
-      <c r="B94" s="1139"/>
+      <c r="A94" s="1156"/>
+      <c r="B94" s="1141"/>
       <c r="C94" s="664">
         <v>7</v>
       </c>
@@ -43184,8 +43184,8 @@
       <c r="M94" s="686"/>
     </row>
     <row r="95" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="1138"/>
-      <c r="B95" s="1139"/>
+      <c r="A95" s="1156"/>
+      <c r="B95" s="1141"/>
       <c r="C95" s="664">
         <v>8</v>
       </c>
@@ -43220,8 +43220,8 @@
       <c r="M95" s="686"/>
     </row>
     <row r="96" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="1138"/>
-      <c r="B96" s="1139"/>
+      <c r="A96" s="1156"/>
+      <c r="B96" s="1141"/>
       <c r="C96" s="664">
         <v>9</v>
       </c>
@@ -43265,8 +43265,8 @@
       <c r="Z96" s="712"/>
     </row>
     <row r="97" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="1138"/>
-      <c r="B97" s="1139"/>
+      <c r="A97" s="1156"/>
+      <c r="B97" s="1141"/>
       <c r="C97" s="664">
         <v>10</v>
       </c>
@@ -43310,8 +43310,8 @@
       <c r="Z97" s="659"/>
     </row>
     <row r="98" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="1138"/>
-      <c r="B98" s="1139"/>
+      <c r="A98" s="1156"/>
+      <c r="B98" s="1141"/>
       <c r="C98" s="664">
         <v>11</v>
       </c>
@@ -43369,8 +43369,8 @@
       </c>
     </row>
     <row r="99" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="1138"/>
-      <c r="B99" s="1139"/>
+      <c r="A99" s="1156"/>
+      <c r="B99" s="1141"/>
       <c r="C99" s="693">
         <v>12</v>
       </c>
@@ -43408,10 +43408,10 @@
       </c>
     </row>
     <row r="100" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A100" s="1150">
+      <c r="A100" s="1154">
         <v>7</v>
       </c>
-      <c r="B100" s="1148">
+      <c r="B100" s="1152">
         <v>2030</v>
       </c>
       <c r="C100" s="660">
@@ -43449,8 +43449,8 @@
       </c>
     </row>
     <row r="101" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A101" s="1150"/>
-      <c r="B101" s="1148"/>
+      <c r="A101" s="1154"/>
+      <c r="B101" s="1152"/>
       <c r="C101" s="664">
         <v>2</v>
       </c>
@@ -43489,8 +43489,8 @@
       </c>
     </row>
     <row r="102" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="1150"/>
-      <c r="B102" s="1148"/>
+      <c r="A102" s="1154"/>
+      <c r="B102" s="1152"/>
       <c r="C102" s="664">
         <v>3</v>
       </c>
@@ -43529,8 +43529,8 @@
       </c>
     </row>
     <row r="103" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A103" s="1150"/>
-      <c r="B103" s="1148"/>
+      <c r="A103" s="1154"/>
+      <c r="B103" s="1152"/>
       <c r="C103" s="664">
         <v>4</v>
       </c>
@@ -43568,8 +43568,8 @@
       </c>
     </row>
     <row r="104" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A104" s="1150"/>
-      <c r="B104" s="1148"/>
+      <c r="A104" s="1154"/>
+      <c r="B104" s="1152"/>
       <c r="C104" s="664">
         <v>5</v>
       </c>
@@ -43607,8 +43607,8 @@
       </c>
     </row>
     <row r="105" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A105" s="1150"/>
-      <c r="B105" s="1148"/>
+      <c r="A105" s="1154"/>
+      <c r="B105" s="1152"/>
       <c r="C105" s="664">
         <v>6</v>
       </c>
@@ -43646,8 +43646,8 @@
       </c>
     </row>
     <row r="106" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A106" s="1150"/>
-      <c r="B106" s="1148"/>
+      <c r="A106" s="1154"/>
+      <c r="B106" s="1152"/>
       <c r="C106" s="664">
         <v>7</v>
       </c>
@@ -43685,8 +43685,8 @@
       </c>
     </row>
     <row r="107" spans="1:26" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A107" s="1151"/>
-      <c r="B107" s="1149"/>
+      <c r="A107" s="1155"/>
+      <c r="B107" s="1153"/>
       <c r="C107" s="664">
         <v>8</v>
       </c>
@@ -43798,6 +43798,23 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A4:A15"/>
+    <mergeCell ref="B4:B15"/>
+    <mergeCell ref="A76:A87"/>
+    <mergeCell ref="B76:B87"/>
+    <mergeCell ref="A88:A99"/>
+    <mergeCell ref="B88:B99"/>
+    <mergeCell ref="A28:A39"/>
+    <mergeCell ref="B28:B39"/>
+    <mergeCell ref="A16:A27"/>
+    <mergeCell ref="B100:B107"/>
+    <mergeCell ref="A100:A107"/>
+    <mergeCell ref="A40:A51"/>
+    <mergeCell ref="B40:B51"/>
+    <mergeCell ref="A52:A63"/>
+    <mergeCell ref="B52:B63"/>
+    <mergeCell ref="A64:A75"/>
+    <mergeCell ref="B64:B75"/>
     <mergeCell ref="P28:V28"/>
     <mergeCell ref="X28:AD28"/>
     <mergeCell ref="AF28:AL28"/>
@@ -43808,23 +43825,6 @@
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="B16:B27"/>
     <mergeCell ref="D1:H1"/>
-    <mergeCell ref="B100:B107"/>
-    <mergeCell ref="A100:A107"/>
-    <mergeCell ref="A40:A51"/>
-    <mergeCell ref="B40:B51"/>
-    <mergeCell ref="A52:A63"/>
-    <mergeCell ref="B52:B63"/>
-    <mergeCell ref="A64:A75"/>
-    <mergeCell ref="B64:B75"/>
-    <mergeCell ref="A4:A15"/>
-    <mergeCell ref="B4:B15"/>
-    <mergeCell ref="A76:A87"/>
-    <mergeCell ref="B76:B87"/>
-    <mergeCell ref="A88:A99"/>
-    <mergeCell ref="B88:B99"/>
-    <mergeCell ref="A28:A39"/>
-    <mergeCell ref="B28:B39"/>
-    <mergeCell ref="A16:A27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>